<commit_message>
Inscrit les encaissements Vinted du 21/08 et du 10/09 : CA du 3e trimestre à 587 €
Salomon X Ultra 5 (100 €, encaissée le 21/08), New Balance GS 1906
Alkaline Green (99 €) et une paire de Havaianas (15 €, encaissées le
10/09) ajoutées au livre des recettes, au registre des objets mobiliers,
à la liste de vente et au stock.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="À vendre" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="À vendre" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -655,7 +655,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>✅ VENDU — 373 € encaissés de clients réels</t>
+          <t>✅ VENDU — 587 € encaissés de clients réels</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -725,7 +725,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Vendue le 12/08 · EXPÉDIÉE le 14/08, locker Mondial Relay · en attente d'encaissement</t>
+          <t>Vendue le 12/08 · expédiée le 14/08 · encaissée le 21/08</t>
         </is>
       </c>
       <c r="H7" s="18" t="n"/>
@@ -1111,7 +1111,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Havaianas Slim fuchsia 35/36 — à l'unité, 10 restantes</t>
+          <t>Havaianas Slim fuchsia 35/36 — à l'unité, 9 restantes</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
+          <t>1 paire vendue 15 € sur Vinted, encaissée le 10/09 · Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
         </is>
       </c>
       <c r="H20" s="12" t="n"/>
@@ -2111,7 +2111,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>New Balance GS 1906 Alkaline Green — 38½</t>
+          <t>✅ VENDUE — New Balance GS 1906 Alkaline Green — 38½</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
@@ -2130,15 +2130,19 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Vinted</t>
         </is>
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>AU-DESSUS du marché 87 € StockX — à trancher</t>
-        </is>
-      </c>
-      <c r="H53" s="12" t="n"/>
+          <t>Vendue 99 € sur Vinted · encaissée le 10/09</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Renseigne les pseudonymes Vinted des acheteurs du 10/09 (Calvimo, amaliagogoi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1135,7 +1135,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>1 paire vendue 15 € sur Vinted, encaissée le 10/09 · Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
+          <t>1 paire vendue 15 € sur Vinted à « amaliagogoi », encaissée le 10/09 · Moins cher du net 15 €/paire · 25 € par vente HORS D'ATTEINTE</t>
         </is>
       </c>
       <c r="H20" s="12" t="n"/>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>Vendue 99 € sur Vinted · encaissée le 10/09</t>
+          <t>Vendue 99 € sur Vinted à « Calvimo » · encaissée le 10/09</t>
         </is>
       </c>
       <c r="H53" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Ballerines Massimo Dutti vendues 50 € le 17/10 sur Vinted, encaissement en attente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wzBucwCEyZdD3ZWCqvChZ
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-liste-de-vente.xlsx
+++ b/exports/maison-nsaia-liste-de-vente.xlsx
@@ -1729,11 +1729,11 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>Ballerines Massimo Dutti cuir rouge — 40 IT</t>
+          <t>✅ VENDUE — Ballerines Massimo Dutti cuir rouge — 40 IT</t>
         </is>
       </c>
       <c r="B40" s="14" t="n">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C40" s="27" t="n">
         <v>25.87</v>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="F40" s="13" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Vinted</t>
         </is>
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>59 → 61 € · marché 70 € · pas Vinted : article neuf</t>
+          <t>Vendue 50 € le 17/10 sur Vinted · en attente d'encaissement</t>
         </is>
       </c>
       <c r="H40" s="18" t="n"/>

</xml_diff>